<commit_message>
Auto: actualizacion datos climaticos
</commit_message>
<xml_diff>
--- a/364053_daily_station_data.xlsx
+++ b/364053_daily_station_data.xlsx
@@ -364,7 +364,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="272">
   <si>
     <t>Time</t>
   </si>
@@ -1114,6 +1114,72 @@
   </si>
   <si>
     <t>2026-10-26 18:30</t>
+  </si>
+  <si>
+    <t>2026-10-26 18:35</t>
+  </si>
+  <si>
+    <t>2026-10-26 18:40</t>
+  </si>
+  <si>
+    <t>2026-10-26 18:45</t>
+  </si>
+  <si>
+    <t>2026-10-26 18:50</t>
+  </si>
+  <si>
+    <t>2026-10-26 18:55</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:00</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:05</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:10</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:15</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:20</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:25</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:30</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:35</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:40</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:45</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:50</t>
+  </si>
+  <si>
+    <t>2026-10-26 19:55</t>
+  </si>
+  <si>
+    <t>2026-10-26 20:00</t>
+  </si>
+  <si>
+    <t>2026-10-26 20:05</t>
+  </si>
+  <si>
+    <t>2026-10-26 20:10</t>
+  </si>
+  <si>
+    <t>2026-10-26 20:15</t>
+  </si>
+  <si>
+    <t>2026-10-26 20:20</t>
   </si>
 </sst>
 </file>
@@ -1701,7 +1767,7 @@
     <tabColor rgb="FF0094FF"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
   </sheetPr>
-  <dimension ref="A1:V224"/>
+  <dimension ref="A1:V246"/>
   <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="21" customWidth="true" style="0"/>
@@ -16859,71 +16925,1567 @@
       </c>
     </row>
     <row r="224" spans="1:22" customHeight="1" ht="18">
-      <c r="A224" s="19" t="s">
+      <c r="A224" s="13" t="s">
         <v>249</v>
       </c>
-      <c r="B224" s="20">
+      <c r="B224" s="14">
         <v>20.4</v>
       </c>
-      <c r="C224" s="20">
+      <c r="C224" s="14">
         <v>20.4</v>
       </c>
-      <c r="D224" s="20">
+      <c r="D224" s="14">
         <v>11.6</v>
       </c>
-      <c r="E224" s="21">
+      <c r="E224" s="15">
         <v>57</v>
       </c>
-      <c r="F224" s="22">
+      <c r="F224" s="16">
         <v>1.029</v>
       </c>
-      <c r="G224" s="20">
-        <v>0</v>
-      </c>
-      <c r="H224" s="21">
-        <v>0</v>
-      </c>
-      <c r="I224" s="20">
-        <v>0</v>
-      </c>
-      <c r="J224" s="20">
-        <v>0</v>
-      </c>
-      <c r="K224" s="20">
-        <v>0</v>
-      </c>
-      <c r="L224" s="20">
-        <v>0</v>
-      </c>
-      <c r="M224" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="N224" s="20">
-        <v>0</v>
-      </c>
-      <c r="O224" s="20">
-        <v>2.8</v>
-      </c>
-      <c r="P224" s="20">
-        <v>2.8</v>
-      </c>
-      <c r="Q224" s="20">
-        <v>0</v>
-      </c>
-      <c r="R224" s="20">
-        <v>0</v>
-      </c>
-      <c r="S224" s="21">
-        <v>55</v>
-      </c>
-      <c r="T224" s="23" t="s">
-        <v>28</v>
-      </c>
-      <c r="U224" s="20">
+      <c r="G224" s="14">
+        <v>0</v>
+      </c>
+      <c r="H224" s="15">
+        <v>0</v>
+      </c>
+      <c r="I224" s="14">
+        <v>0</v>
+      </c>
+      <c r="J224" s="14">
+        <v>0</v>
+      </c>
+      <c r="K224" s="14">
+        <v>0</v>
+      </c>
+      <c r="L224" s="14">
+        <v>0</v>
+      </c>
+      <c r="M224" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N224" s="14">
+        <v>0</v>
+      </c>
+      <c r="O224" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P224" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q224" s="14">
+        <v>0</v>
+      </c>
+      <c r="R224" s="14">
+        <v>0</v>
+      </c>
+      <c r="S224" s="15">
+        <v>55</v>
+      </c>
+      <c r="T224" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U224" s="14">
         <v>1019.4</v>
       </c>
-      <c r="V224" s="24">
+      <c r="V224" s="18">
         <v>876.7</v>
+      </c>
+    </row>
+    <row r="225" spans="1:22" customHeight="1" ht="18">
+      <c r="A225" s="2" t="s">
+        <v>250</v>
+      </c>
+      <c r="B225" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C225" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D225" s="7">
+        <v>11.6</v>
+      </c>
+      <c r="E225" s="8">
+        <v>57</v>
+      </c>
+      <c r="F225" s="9">
+        <v>1.029</v>
+      </c>
+      <c r="G225" s="7">
+        <v>0</v>
+      </c>
+      <c r="H225" s="8">
+        <v>0</v>
+      </c>
+      <c r="I225" s="7">
+        <v>0</v>
+      </c>
+      <c r="J225" s="7">
+        <v>0</v>
+      </c>
+      <c r="K225" s="7">
+        <v>0</v>
+      </c>
+      <c r="L225" s="7">
+        <v>0</v>
+      </c>
+      <c r="M225" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N225" s="7">
+        <v>0</v>
+      </c>
+      <c r="O225" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P225" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q225" s="7">
+        <v>0</v>
+      </c>
+      <c r="R225" s="7">
+        <v>0</v>
+      </c>
+      <c r="S225" s="8">
+        <v>55</v>
+      </c>
+      <c r="T225" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U225" s="7">
+        <v>1019.9</v>
+      </c>
+      <c r="V225" s="12">
+        <v>877.2</v>
+      </c>
+    </row>
+    <row r="226" spans="1:22" customHeight="1" ht="18">
+      <c r="A226" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="B226" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C226" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D226" s="14">
+        <v>11.6</v>
+      </c>
+      <c r="E226" s="15">
+        <v>57</v>
+      </c>
+      <c r="F226" s="16">
+        <v>1.029</v>
+      </c>
+      <c r="G226" s="14">
+        <v>0</v>
+      </c>
+      <c r="H226" s="15">
+        <v>0</v>
+      </c>
+      <c r="I226" s="14">
+        <v>0</v>
+      </c>
+      <c r="J226" s="14">
+        <v>0</v>
+      </c>
+      <c r="K226" s="14">
+        <v>0</v>
+      </c>
+      <c r="L226" s="14">
+        <v>0</v>
+      </c>
+      <c r="M226" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N226" s="14">
+        <v>0</v>
+      </c>
+      <c r="O226" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P226" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q226" s="14">
+        <v>0</v>
+      </c>
+      <c r="R226" s="14">
+        <v>0</v>
+      </c>
+      <c r="S226" s="15">
+        <v>55</v>
+      </c>
+      <c r="T226" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U226" s="14">
+        <v>1019.9</v>
+      </c>
+      <c r="V226" s="18">
+        <v>877.2</v>
+      </c>
+    </row>
+    <row r="227" spans="1:22" customHeight="1" ht="18">
+      <c r="A227" s="2" t="s">
+        <v>252</v>
+      </c>
+      <c r="B227" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C227" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D227" s="7">
+        <v>11.6</v>
+      </c>
+      <c r="E227" s="8">
+        <v>57</v>
+      </c>
+      <c r="F227" s="9">
+        <v>1.029</v>
+      </c>
+      <c r="G227" s="7">
+        <v>0</v>
+      </c>
+      <c r="H227" s="8">
+        <v>0</v>
+      </c>
+      <c r="I227" s="7">
+        <v>0</v>
+      </c>
+      <c r="J227" s="7">
+        <v>0</v>
+      </c>
+      <c r="K227" s="7">
+        <v>0</v>
+      </c>
+      <c r="L227" s="7">
+        <v>0</v>
+      </c>
+      <c r="M227" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N227" s="7">
+        <v>0</v>
+      </c>
+      <c r="O227" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P227" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q227" s="7">
+        <v>0</v>
+      </c>
+      <c r="R227" s="7">
+        <v>0</v>
+      </c>
+      <c r="S227" s="8">
+        <v>55</v>
+      </c>
+      <c r="T227" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U227" s="7">
+        <v>1019.9</v>
+      </c>
+      <c r="V227" s="12">
+        <v>877.2</v>
+      </c>
+    </row>
+    <row r="228" spans="1:22" customHeight="1" ht="18">
+      <c r="A228" s="13" t="s">
+        <v>253</v>
+      </c>
+      <c r="B228" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C228" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D228" s="14">
+        <v>11.6</v>
+      </c>
+      <c r="E228" s="15">
+        <v>57</v>
+      </c>
+      <c r="F228" s="16">
+        <v>1.029</v>
+      </c>
+      <c r="G228" s="14">
+        <v>0</v>
+      </c>
+      <c r="H228" s="15">
+        <v>0</v>
+      </c>
+      <c r="I228" s="14">
+        <v>0</v>
+      </c>
+      <c r="J228" s="14">
+        <v>0</v>
+      </c>
+      <c r="K228" s="14">
+        <v>0</v>
+      </c>
+      <c r="L228" s="14">
+        <v>0</v>
+      </c>
+      <c r="M228" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N228" s="14">
+        <v>0</v>
+      </c>
+      <c r="O228" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P228" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q228" s="14">
+        <v>0</v>
+      </c>
+      <c r="R228" s="14">
+        <v>0</v>
+      </c>
+      <c r="S228" s="15">
+        <v>55</v>
+      </c>
+      <c r="T228" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U228" s="14">
+        <v>1020.1</v>
+      </c>
+      <c r="V228" s="18">
+        <v>877.4</v>
+      </c>
+    </row>
+    <row r="229" spans="1:22" customHeight="1" ht="18">
+      <c r="A229" s="2" t="s">
+        <v>254</v>
+      </c>
+      <c r="B229" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C229" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D229" s="7">
+        <v>11.6</v>
+      </c>
+      <c r="E229" s="8">
+        <v>57</v>
+      </c>
+      <c r="F229" s="9">
+        <v>1.029</v>
+      </c>
+      <c r="G229" s="7">
+        <v>0</v>
+      </c>
+      <c r="H229" s="8">
+        <v>0</v>
+      </c>
+      <c r="I229" s="7">
+        <v>0</v>
+      </c>
+      <c r="J229" s="7">
+        <v>0</v>
+      </c>
+      <c r="K229" s="7">
+        <v>0</v>
+      </c>
+      <c r="L229" s="7">
+        <v>0</v>
+      </c>
+      <c r="M229" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N229" s="7">
+        <v>0</v>
+      </c>
+      <c r="O229" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P229" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q229" s="7">
+        <v>0</v>
+      </c>
+      <c r="R229" s="7">
+        <v>0</v>
+      </c>
+      <c r="S229" s="8">
+        <v>55</v>
+      </c>
+      <c r="T229" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U229" s="7">
+        <v>1020.2</v>
+      </c>
+      <c r="V229" s="12">
+        <v>877.5</v>
+      </c>
+    </row>
+    <row r="230" spans="1:22" customHeight="1" ht="18">
+      <c r="A230" s="13" t="s">
+        <v>255</v>
+      </c>
+      <c r="B230" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C230" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D230" s="14">
+        <v>11.6</v>
+      </c>
+      <c r="E230" s="15">
+        <v>57</v>
+      </c>
+      <c r="F230" s="16">
+        <v>1.029</v>
+      </c>
+      <c r="G230" s="14">
+        <v>0</v>
+      </c>
+      <c r="H230" s="15">
+        <v>0</v>
+      </c>
+      <c r="I230" s="14">
+        <v>0</v>
+      </c>
+      <c r="J230" s="14">
+        <v>0</v>
+      </c>
+      <c r="K230" s="14">
+        <v>0</v>
+      </c>
+      <c r="L230" s="14">
+        <v>0</v>
+      </c>
+      <c r="M230" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N230" s="14">
+        <v>0</v>
+      </c>
+      <c r="O230" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P230" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q230" s="14">
+        <v>0</v>
+      </c>
+      <c r="R230" s="14">
+        <v>0</v>
+      </c>
+      <c r="S230" s="15">
+        <v>55</v>
+      </c>
+      <c r="T230" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U230" s="14">
+        <v>1020.2</v>
+      </c>
+      <c r="V230" s="18">
+        <v>877.5</v>
+      </c>
+    </row>
+    <row r="231" spans="1:22" customHeight="1" ht="18">
+      <c r="A231" s="2" t="s">
+        <v>256</v>
+      </c>
+      <c r="B231" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C231" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D231" s="7">
+        <v>11.6</v>
+      </c>
+      <c r="E231" s="8">
+        <v>57</v>
+      </c>
+      <c r="F231" s="9">
+        <v>1.029</v>
+      </c>
+      <c r="G231" s="7">
+        <v>0</v>
+      </c>
+      <c r="H231" s="8">
+        <v>0</v>
+      </c>
+      <c r="I231" s="7">
+        <v>0</v>
+      </c>
+      <c r="J231" s="7">
+        <v>0</v>
+      </c>
+      <c r="K231" s="7">
+        <v>0</v>
+      </c>
+      <c r="L231" s="7">
+        <v>0</v>
+      </c>
+      <c r="M231" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N231" s="7">
+        <v>0</v>
+      </c>
+      <c r="O231" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P231" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q231" s="7">
+        <v>0</v>
+      </c>
+      <c r="R231" s="7">
+        <v>0</v>
+      </c>
+      <c r="S231" s="8">
+        <v>55</v>
+      </c>
+      <c r="T231" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U231" s="7">
+        <v>1020.2</v>
+      </c>
+      <c r="V231" s="12">
+        <v>877.5</v>
+      </c>
+    </row>
+    <row r="232" spans="1:22" customHeight="1" ht="18">
+      <c r="A232" s="13" t="s">
+        <v>257</v>
+      </c>
+      <c r="B232" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C232" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D232" s="14">
+        <v>11.6</v>
+      </c>
+      <c r="E232" s="15">
+        <v>57</v>
+      </c>
+      <c r="F232" s="16">
+        <v>1.029</v>
+      </c>
+      <c r="G232" s="14">
+        <v>0</v>
+      </c>
+      <c r="H232" s="15">
+        <v>0</v>
+      </c>
+      <c r="I232" s="14">
+        <v>0</v>
+      </c>
+      <c r="J232" s="14">
+        <v>0</v>
+      </c>
+      <c r="K232" s="14">
+        <v>0</v>
+      </c>
+      <c r="L232" s="14">
+        <v>0</v>
+      </c>
+      <c r="M232" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N232" s="14">
+        <v>0</v>
+      </c>
+      <c r="O232" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P232" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q232" s="14">
+        <v>0</v>
+      </c>
+      <c r="R232" s="14">
+        <v>0</v>
+      </c>
+      <c r="S232" s="15">
+        <v>55</v>
+      </c>
+      <c r="T232" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U232" s="14">
+        <v>1020.5</v>
+      </c>
+      <c r="V232" s="18">
+        <v>877.8</v>
+      </c>
+    </row>
+    <row r="233" spans="1:22" customHeight="1" ht="18">
+      <c r="A233" s="2" t="s">
+        <v>258</v>
+      </c>
+      <c r="B233" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C233" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D233" s="7">
+        <v>11.6</v>
+      </c>
+      <c r="E233" s="8">
+        <v>57</v>
+      </c>
+      <c r="F233" s="9">
+        <v>1.029</v>
+      </c>
+      <c r="G233" s="7">
+        <v>0</v>
+      </c>
+      <c r="H233" s="8">
+        <v>0</v>
+      </c>
+      <c r="I233" s="7">
+        <v>0</v>
+      </c>
+      <c r="J233" s="7">
+        <v>0</v>
+      </c>
+      <c r="K233" s="7">
+        <v>0</v>
+      </c>
+      <c r="L233" s="7">
+        <v>0</v>
+      </c>
+      <c r="M233" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N233" s="7">
+        <v>0</v>
+      </c>
+      <c r="O233" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P233" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q233" s="7">
+        <v>0</v>
+      </c>
+      <c r="R233" s="7">
+        <v>0</v>
+      </c>
+      <c r="S233" s="8">
+        <v>55</v>
+      </c>
+      <c r="T233" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U233" s="7">
+        <v>1020.5</v>
+      </c>
+      <c r="V233" s="12">
+        <v>877.8</v>
+      </c>
+    </row>
+    <row r="234" spans="1:22" customHeight="1" ht="18">
+      <c r="A234" s="13" t="s">
+        <v>259</v>
+      </c>
+      <c r="B234" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C234" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D234" s="14">
+        <v>11.6</v>
+      </c>
+      <c r="E234" s="15">
+        <v>57</v>
+      </c>
+      <c r="F234" s="16">
+        <v>1.029</v>
+      </c>
+      <c r="G234" s="14">
+        <v>0</v>
+      </c>
+      <c r="H234" s="15">
+        <v>0</v>
+      </c>
+      <c r="I234" s="14">
+        <v>0</v>
+      </c>
+      <c r="J234" s="14">
+        <v>0</v>
+      </c>
+      <c r="K234" s="14">
+        <v>0</v>
+      </c>
+      <c r="L234" s="14">
+        <v>0</v>
+      </c>
+      <c r="M234" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N234" s="14">
+        <v>0</v>
+      </c>
+      <c r="O234" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P234" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q234" s="14">
+        <v>0</v>
+      </c>
+      <c r="R234" s="14">
+        <v>0</v>
+      </c>
+      <c r="S234" s="15">
+        <v>55</v>
+      </c>
+      <c r="T234" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U234" s="14">
+        <v>1020.4</v>
+      </c>
+      <c r="V234" s="18">
+        <v>877.7</v>
+      </c>
+    </row>
+    <row r="235" spans="1:22" customHeight="1" ht="18">
+      <c r="A235" s="2" t="s">
+        <v>260</v>
+      </c>
+      <c r="B235" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C235" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D235" s="7">
+        <v>11.6</v>
+      </c>
+      <c r="E235" s="8">
+        <v>57</v>
+      </c>
+      <c r="F235" s="9">
+        <v>1.029</v>
+      </c>
+      <c r="G235" s="7">
+        <v>0</v>
+      </c>
+      <c r="H235" s="8">
+        <v>0</v>
+      </c>
+      <c r="I235" s="7">
+        <v>0</v>
+      </c>
+      <c r="J235" s="7">
+        <v>0</v>
+      </c>
+      <c r="K235" s="7">
+        <v>0</v>
+      </c>
+      <c r="L235" s="7">
+        <v>0</v>
+      </c>
+      <c r="M235" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N235" s="7">
+        <v>0</v>
+      </c>
+      <c r="O235" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P235" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q235" s="7">
+        <v>0</v>
+      </c>
+      <c r="R235" s="7">
+        <v>0</v>
+      </c>
+      <c r="S235" s="8">
+        <v>55</v>
+      </c>
+      <c r="T235" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U235" s="7">
+        <v>1020.4</v>
+      </c>
+      <c r="V235" s="12">
+        <v>877.7</v>
+      </c>
+    </row>
+    <row r="236" spans="1:22" customHeight="1" ht="18">
+      <c r="A236" s="13" t="s">
+        <v>261</v>
+      </c>
+      <c r="B236" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C236" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D236" s="14">
+        <v>11.8</v>
+      </c>
+      <c r="E236" s="15">
+        <v>58</v>
+      </c>
+      <c r="F236" s="16">
+        <v>1.006</v>
+      </c>
+      <c r="G236" s="14">
+        <v>0</v>
+      </c>
+      <c r="H236" s="15">
+        <v>0</v>
+      </c>
+      <c r="I236" s="14">
+        <v>0</v>
+      </c>
+      <c r="J236" s="14">
+        <v>0</v>
+      </c>
+      <c r="K236" s="14">
+        <v>0</v>
+      </c>
+      <c r="L236" s="14">
+        <v>0</v>
+      </c>
+      <c r="M236" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N236" s="14">
+        <v>0</v>
+      </c>
+      <c r="O236" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P236" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q236" s="14">
+        <v>0</v>
+      </c>
+      <c r="R236" s="14">
+        <v>0</v>
+      </c>
+      <c r="S236" s="15">
+        <v>55</v>
+      </c>
+      <c r="T236" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U236" s="14">
+        <v>1020.6</v>
+      </c>
+      <c r="V236" s="18">
+        <v>877.9</v>
+      </c>
+    </row>
+    <row r="237" spans="1:22" customHeight="1" ht="18">
+      <c r="A237" s="2" t="s">
+        <v>262</v>
+      </c>
+      <c r="B237" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C237" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D237" s="7">
+        <v>11.8</v>
+      </c>
+      <c r="E237" s="8">
+        <v>58</v>
+      </c>
+      <c r="F237" s="9">
+        <v>1.006</v>
+      </c>
+      <c r="G237" s="7">
+        <v>0</v>
+      </c>
+      <c r="H237" s="8">
+        <v>0</v>
+      </c>
+      <c r="I237" s="7">
+        <v>0</v>
+      </c>
+      <c r="J237" s="7">
+        <v>0</v>
+      </c>
+      <c r="K237" s="7">
+        <v>0</v>
+      </c>
+      <c r="L237" s="7">
+        <v>0</v>
+      </c>
+      <c r="M237" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N237" s="7">
+        <v>0</v>
+      </c>
+      <c r="O237" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P237" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q237" s="7">
+        <v>0</v>
+      </c>
+      <c r="R237" s="7">
+        <v>0</v>
+      </c>
+      <c r="S237" s="8">
+        <v>55</v>
+      </c>
+      <c r="T237" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U237" s="7">
+        <v>1020.5</v>
+      </c>
+      <c r="V237" s="12">
+        <v>877.8</v>
+      </c>
+    </row>
+    <row r="238" spans="1:22" customHeight="1" ht="18">
+      <c r="A238" s="13" t="s">
+        <v>263</v>
+      </c>
+      <c r="B238" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C238" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D238" s="14">
+        <v>11.6</v>
+      </c>
+      <c r="E238" s="15">
+        <v>57</v>
+      </c>
+      <c r="F238" s="16">
+        <v>1.029</v>
+      </c>
+      <c r="G238" s="14">
+        <v>0</v>
+      </c>
+      <c r="H238" s="15">
+        <v>0</v>
+      </c>
+      <c r="I238" s="14">
+        <v>0</v>
+      </c>
+      <c r="J238" s="14">
+        <v>0</v>
+      </c>
+      <c r="K238" s="14">
+        <v>0</v>
+      </c>
+      <c r="L238" s="14">
+        <v>0</v>
+      </c>
+      <c r="M238" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N238" s="14">
+        <v>0</v>
+      </c>
+      <c r="O238" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P238" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q238" s="14">
+        <v>0</v>
+      </c>
+      <c r="R238" s="14">
+        <v>0</v>
+      </c>
+      <c r="S238" s="15">
+        <v>55</v>
+      </c>
+      <c r="T238" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U238" s="14">
+        <v>1020.7</v>
+      </c>
+      <c r="V238" s="18">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="239" spans="1:22" customHeight="1" ht="18">
+      <c r="A239" s="2" t="s">
+        <v>264</v>
+      </c>
+      <c r="B239" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C239" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D239" s="7">
+        <v>11.8</v>
+      </c>
+      <c r="E239" s="8">
+        <v>58</v>
+      </c>
+      <c r="F239" s="9">
+        <v>1.006</v>
+      </c>
+      <c r="G239" s="7">
+        <v>0</v>
+      </c>
+      <c r="H239" s="8">
+        <v>0</v>
+      </c>
+      <c r="I239" s="7">
+        <v>0</v>
+      </c>
+      <c r="J239" s="7">
+        <v>0</v>
+      </c>
+      <c r="K239" s="7">
+        <v>0</v>
+      </c>
+      <c r="L239" s="7">
+        <v>0</v>
+      </c>
+      <c r="M239" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N239" s="7">
+        <v>0</v>
+      </c>
+      <c r="O239" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P239" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q239" s="7">
+        <v>0</v>
+      </c>
+      <c r="R239" s="7">
+        <v>0</v>
+      </c>
+      <c r="S239" s="8">
+        <v>55</v>
+      </c>
+      <c r="T239" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U239" s="7">
+        <v>1020.5</v>
+      </c>
+      <c r="V239" s="12">
+        <v>877.8</v>
+      </c>
+    </row>
+    <row r="240" spans="1:22" customHeight="1" ht="18">
+      <c r="A240" s="13" t="s">
+        <v>265</v>
+      </c>
+      <c r="B240" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C240" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D240" s="14">
+        <v>11.8</v>
+      </c>
+      <c r="E240" s="15">
+        <v>58</v>
+      </c>
+      <c r="F240" s="16">
+        <v>1.006</v>
+      </c>
+      <c r="G240" s="14">
+        <v>0</v>
+      </c>
+      <c r="H240" s="15">
+        <v>0</v>
+      </c>
+      <c r="I240" s="14">
+        <v>0</v>
+      </c>
+      <c r="J240" s="14">
+        <v>0</v>
+      </c>
+      <c r="K240" s="14">
+        <v>0</v>
+      </c>
+      <c r="L240" s="14">
+        <v>0</v>
+      </c>
+      <c r="M240" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N240" s="14">
+        <v>0</v>
+      </c>
+      <c r="O240" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P240" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q240" s="14">
+        <v>0</v>
+      </c>
+      <c r="R240" s="14">
+        <v>0</v>
+      </c>
+      <c r="S240" s="15">
+        <v>55</v>
+      </c>
+      <c r="T240" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U240" s="14">
+        <v>1020.8</v>
+      </c>
+      <c r="V240" s="18">
+        <v>878.1</v>
+      </c>
+    </row>
+    <row r="241" spans="1:22" customHeight="1" ht="18">
+      <c r="A241" s="2" t="s">
+        <v>266</v>
+      </c>
+      <c r="B241" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C241" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D241" s="7">
+        <v>11.8</v>
+      </c>
+      <c r="E241" s="8">
+        <v>58</v>
+      </c>
+      <c r="F241" s="9">
+        <v>1.006</v>
+      </c>
+      <c r="G241" s="7">
+        <v>0</v>
+      </c>
+      <c r="H241" s="8">
+        <v>0</v>
+      </c>
+      <c r="I241" s="7">
+        <v>0</v>
+      </c>
+      <c r="J241" s="7">
+        <v>0</v>
+      </c>
+      <c r="K241" s="7">
+        <v>0</v>
+      </c>
+      <c r="L241" s="7">
+        <v>0</v>
+      </c>
+      <c r="M241" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N241" s="7">
+        <v>0</v>
+      </c>
+      <c r="O241" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P241" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q241" s="7">
+        <v>0</v>
+      </c>
+      <c r="R241" s="7">
+        <v>0</v>
+      </c>
+      <c r="S241" s="8">
+        <v>55</v>
+      </c>
+      <c r="T241" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U241" s="7">
+        <v>1020.7</v>
+      </c>
+      <c r="V241" s="12">
+        <v>878</v>
+      </c>
+    </row>
+    <row r="242" spans="1:22" customHeight="1" ht="18">
+      <c r="A242" s="13" t="s">
+        <v>267</v>
+      </c>
+      <c r="B242" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C242" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D242" s="14">
+        <v>11.8</v>
+      </c>
+      <c r="E242" s="15">
+        <v>58</v>
+      </c>
+      <c r="F242" s="16">
+        <v>1.006</v>
+      </c>
+      <c r="G242" s="14">
+        <v>0</v>
+      </c>
+      <c r="H242" s="15">
+        <v>0</v>
+      </c>
+      <c r="I242" s="14">
+        <v>0</v>
+      </c>
+      <c r="J242" s="14">
+        <v>0</v>
+      </c>
+      <c r="K242" s="14">
+        <v>0</v>
+      </c>
+      <c r="L242" s="14">
+        <v>0</v>
+      </c>
+      <c r="M242" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N242" s="14">
+        <v>0</v>
+      </c>
+      <c r="O242" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P242" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q242" s="14">
+        <v>0</v>
+      </c>
+      <c r="R242" s="14">
+        <v>0</v>
+      </c>
+      <c r="S242" s="15">
+        <v>55</v>
+      </c>
+      <c r="T242" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U242" s="14">
+        <v>1020.5</v>
+      </c>
+      <c r="V242" s="18">
+        <v>877.8</v>
+      </c>
+    </row>
+    <row r="243" spans="1:22" customHeight="1" ht="18">
+      <c r="A243" s="2" t="s">
+        <v>268</v>
+      </c>
+      <c r="B243" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C243" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D243" s="7">
+        <v>11.8</v>
+      </c>
+      <c r="E243" s="8">
+        <v>58</v>
+      </c>
+      <c r="F243" s="9">
+        <v>1.006</v>
+      </c>
+      <c r="G243" s="7">
+        <v>0</v>
+      </c>
+      <c r="H243" s="8">
+        <v>0</v>
+      </c>
+      <c r="I243" s="7">
+        <v>0</v>
+      </c>
+      <c r="J243" s="7">
+        <v>0</v>
+      </c>
+      <c r="K243" s="7">
+        <v>0</v>
+      </c>
+      <c r="L243" s="7">
+        <v>0</v>
+      </c>
+      <c r="M243" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N243" s="7">
+        <v>0</v>
+      </c>
+      <c r="O243" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P243" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q243" s="7">
+        <v>0</v>
+      </c>
+      <c r="R243" s="7">
+        <v>0</v>
+      </c>
+      <c r="S243" s="8">
+        <v>55</v>
+      </c>
+      <c r="T243" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U243" s="7">
+        <v>1020.5</v>
+      </c>
+      <c r="V243" s="12">
+        <v>877.8</v>
+      </c>
+    </row>
+    <row r="244" spans="1:22" customHeight="1" ht="18">
+      <c r="A244" s="13" t="s">
+        <v>269</v>
+      </c>
+      <c r="B244" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="C244" s="14">
+        <v>20.4</v>
+      </c>
+      <c r="D244" s="14">
+        <v>11.8</v>
+      </c>
+      <c r="E244" s="15">
+        <v>58</v>
+      </c>
+      <c r="F244" s="16">
+        <v>1.006</v>
+      </c>
+      <c r="G244" s="14">
+        <v>0</v>
+      </c>
+      <c r="H244" s="15">
+        <v>0</v>
+      </c>
+      <c r="I244" s="14">
+        <v>0</v>
+      </c>
+      <c r="J244" s="14">
+        <v>0</v>
+      </c>
+      <c r="K244" s="14">
+        <v>0</v>
+      </c>
+      <c r="L244" s="14">
+        <v>0</v>
+      </c>
+      <c r="M244" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="N244" s="14">
+        <v>0</v>
+      </c>
+      <c r="O244" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="P244" s="14">
+        <v>2.8</v>
+      </c>
+      <c r="Q244" s="14">
+        <v>0</v>
+      </c>
+      <c r="R244" s="14">
+        <v>0</v>
+      </c>
+      <c r="S244" s="15">
+        <v>55</v>
+      </c>
+      <c r="T244" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="U244" s="14">
+        <v>1020.6</v>
+      </c>
+      <c r="V244" s="18">
+        <v>877.9</v>
+      </c>
+    </row>
+    <row r="245" spans="1:22" customHeight="1" ht="18">
+      <c r="A245" s="2" t="s">
+        <v>270</v>
+      </c>
+      <c r="B245" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="C245" s="7">
+        <v>20.4</v>
+      </c>
+      <c r="D245" s="7">
+        <v>11.8</v>
+      </c>
+      <c r="E245" s="8">
+        <v>58</v>
+      </c>
+      <c r="F245" s="9">
+        <v>1.006</v>
+      </c>
+      <c r="G245" s="7">
+        <v>0</v>
+      </c>
+      <c r="H245" s="8">
+        <v>0</v>
+      </c>
+      <c r="I245" s="7">
+        <v>0</v>
+      </c>
+      <c r="J245" s="7">
+        <v>0</v>
+      </c>
+      <c r="K245" s="7">
+        <v>0</v>
+      </c>
+      <c r="L245" s="7">
+        <v>0</v>
+      </c>
+      <c r="M245" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="N245" s="7">
+        <v>0</v>
+      </c>
+      <c r="O245" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="P245" s="7">
+        <v>2.8</v>
+      </c>
+      <c r="Q245" s="7">
+        <v>0</v>
+      </c>
+      <c r="R245" s="7">
+        <v>0</v>
+      </c>
+      <c r="S245" s="8">
+        <v>55</v>
+      </c>
+      <c r="T245" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="U245" s="7">
+        <v>1020.6</v>
+      </c>
+      <c r="V245" s="12">
+        <v>877.9</v>
+      </c>
+    </row>
+    <row r="246" spans="1:22" customHeight="1" ht="18">
+      <c r="A246" s="19" t="s">
+        <v>271</v>
+      </c>
+      <c r="B246" s="20">
+        <v>20.4</v>
+      </c>
+      <c r="C246" s="20">
+        <v>20.4</v>
+      </c>
+      <c r="D246" s="20">
+        <v>11.8</v>
+      </c>
+      <c r="E246" s="21">
+        <v>58</v>
+      </c>
+      <c r="F246" s="22">
+        <v>1.006</v>
+      </c>
+      <c r="G246" s="20">
+        <v>0</v>
+      </c>
+      <c r="H246" s="21">
+        <v>0</v>
+      </c>
+      <c r="I246" s="20">
+        <v>0</v>
+      </c>
+      <c r="J246" s="20">
+        <v>0</v>
+      </c>
+      <c r="K246" s="20">
+        <v>0</v>
+      </c>
+      <c r="L246" s="20">
+        <v>0</v>
+      </c>
+      <c r="M246" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="N246" s="20">
+        <v>0</v>
+      </c>
+      <c r="O246" s="20">
+        <v>2.8</v>
+      </c>
+      <c r="P246" s="20">
+        <v>2.8</v>
+      </c>
+      <c r="Q246" s="20">
+        <v>0</v>
+      </c>
+      <c r="R246" s="20">
+        <v>0</v>
+      </c>
+      <c r="S246" s="21">
+        <v>55</v>
+      </c>
+      <c r="T246" s="23" t="s">
+        <v>28</v>
+      </c>
+      <c r="U246" s="20">
+        <v>1020.7</v>
+      </c>
+      <c r="V246" s="24">
+        <v>878</v>
       </c>
     </row>
   </sheetData>

</xml_diff>